<commit_message>
Templates carry the optional fields, and guard the owner block
Residents now ships with Blood Group, Emergency Contact, Vehicle No,
Vehicle Type, Parking Slot, Profession, Language, Occupants and Pets
alongside the owner columns, and a _Private sheet holds dates of birth,
medical notes, lease dates and police verification — never published,
because of the leading underscore.

The example rows show a tenanted flat with the owner columns filled and
an owner-occupied one with them blank, since that difference is what
decides whether the Owner details button appears at all.

test/cards.test.mjs now asserts the owner block renders, its number is
tappable, it does not steal the resident's own call button, and it stays
away when those columns are empty. It sits after the action row, so a
change to detail rendering could drop it without anything else failing.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/alumni-template.xlsx
+++ b/template/alumni-template.xlsx
@@ -859,7 +859,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C14"/>
+  <dimension ref="A1:C18"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="70.83203125" customWidth="1"/>
@@ -1011,18 +1011,62 @@
     </row>
     <row r="14">
       <c r="A14" t="str">
+        <v>Blood group</v>
+      </c>
+      <c r="B14" t="str">
+        <v>Shown as a red badge on the card. Use a dropdown in your form so you do not collect "o positive" and "O +ve".</v>
+      </c>
+      <c r="C14" t="str">
+        <v>कार्ड पर लाल बैज में दिखता है। फ़ॉर्म में ड्रॉपडाउन रखें।</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>Optional fields</v>
+      </c>
+      <c r="B15" t="str">
+        <v>The first two extra columns show on the card; the rest fold behind a More details button. Search still finds them and opens the card.</v>
+      </c>
+      <c r="C15" t="str">
+        <v>पहले दो अतिरिक्त कॉलम कार्ड पर दिखते हैं, बाक़ी "More details" के पीछे। खोज उन्हें भी ढूँढ लेती है।</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>Owner columns</v>
+      </c>
+      <c r="B16" t="str">
+        <v>Fill Owner Name / Owner Phone / Owner Address only for tenanted flats. They appear behind an Owner details button; leave blank and nothing is shown.</v>
+      </c>
+      <c r="C16" t="str">
+        <v>किरायेदार वाले फ्लैट के लिए ही भरें। खाली छोड़ने पर कुछ नहीं दिखेगा।</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>_Private sheet</v>
+      </c>
+      <c r="B17" t="str">
+        <v>Dates of birth, medical notes, lease dates and police verification live here. The leading underscore keeps the sheet off the website entirely.</v>
+      </c>
+      <c r="C17" t="str">
+        <v>जन्मतिथि, चिकित्सा जानकारी आदि यहाँ रखें। यह शीट वेबसाइट पर कभी नहीं दिखती।</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
         <v>Examples</v>
       </c>
-      <c r="B14" t="str">
+      <c r="B18" t="str">
         <v>Delete the example rows before publishing.</v>
       </c>
-      <c r="C14" t="str">
+      <c r="C18" t="str">
         <v>प्रकाशित करने से पहले उदाहरण पंक्तियाँ हटा दें।</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C14"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C18"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>